<commit_message>
fix: derive week 10 constraints and week 4 cohort state
</commit_message>
<xml_diff>
--- a/halden-week10-data-package/faculty/halden_week10_FACULTY_SOLUTION.xlsx
+++ b/halden-week10-data-package/faculty/halden_week10_FACULTY_SOLUTION.xlsx
@@ -125,7 +125,7 @@
     <t xml:space="preserve">cooperative</t>
   </si>
   <si>
-    <t xml:space="preserve">Stayed liquid in Wk6; wide Wk5 mandate; marginal-cost TP in Wk4; managed the JV partner; read Wk8 well</t>
+    <t xml:space="preserve">Stayed liquid in Wk6; wide Wk5 mandate; Wk4 transfer price left refining reporting below target so Delacroix has no cover; managed the JV partner; read Wk8 well</t>
   </si>
   <si>
     <t xml:space="preserve">reference_constrained</t>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">strained</t>
   </si>
   <si>
-    <t xml:space="preserve">Funded Helix in Wk6; narrow Wk5 mandate; market-based TP in Wk4; burned the JV partner; misread Wk8</t>
+    <t xml:space="preserve">Funded Helix in Wk6; narrow Wk5 mandate; Wk4 transfer price gave refining an above-target windfall (marginal-cost or lazy) so Delacroix has cover; burned the JV partner; misread Wk8</t>
   </si>
   <si>
     <t xml:space="preserve">Worked Example — solved on adjacent data. Study the method, then do Your Analysis.</t>

</xml_diff>